<commit_message>
Agregar columna "granel" al importar productos desde Excel
Antes solo se podian crear productos a granel (venta por gramos) uno por
uno desde la pantalla. Ahora el Excel de importacion acepta una columna
opcional "granel" (si/no) -- si se marca, el precio y el stock de esa
fila se guardan como precio por gramo y stock en gramos, igual que hace
el formulario manual. Se actualizo tambien la plantilla descargable con
un ejemplo.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/web/public/plantillas/plantilla-productos.xlsx
+++ b/web/public/plantillas/plantilla-productos.xlsx
@@ -397,16 +397,17 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H4"/>
+  <dimension ref="A1:I5"/>
   <cols>
-    <col min="1" max="1" width="22.83203125" customWidth="1"/>
-    <col min="2" max="2" width="16.83203125" customWidth="1"/>
+    <col min="1" max="1" width="28.83203125" customWidth="1"/>
+    <col min="2" max="2" width="14.83203125" customWidth="1"/>
     <col min="3" max="3" width="10.83203125" customWidth="1"/>
     <col min="4" max="4" width="10.83203125" customWidth="1"/>
-    <col min="5" max="5" width="8.83203125" customWidth="1"/>
+    <col min="5" max="5" width="10.83203125" customWidth="1"/>
     <col min="6" max="6" width="12.83203125" customWidth="1"/>
-    <col min="7" max="7" width="16.83203125" customWidth="1"/>
-    <col min="8" max="8" width="26.83203125" customWidth="1"/>
+    <col min="7" max="7" width="18.83203125" customWidth="1"/>
+    <col min="8" max="8" width="24.83203125" customWidth="1"/>
+    <col min="9" max="9" width="8.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -434,6 +435,9 @@
       <c r="H1" t="str">
         <v>descripcion</v>
       </c>
+      <c r="I1" t="str">
+        <v>granel</v>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="str">
@@ -460,6 +464,9 @@
       <c r="H2" t="str">
         <v>Gaseosa personal</v>
       </c>
+      <c r="I2" t="str">
+        <v/>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
@@ -486,6 +493,9 @@
       <c r="H3" t="str">
         <v>Arroz blanco</v>
       </c>
+      <c r="I3" t="str">
+        <v/>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
@@ -512,10 +522,42 @@
       <c r="H4" t="str">
         <v/>
       </c>
+      <c r="I4" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="str">
+        <v>Maíz Morado</v>
+      </c>
+      <c r="B5" t="str">
+        <v>Granel</v>
+      </c>
+      <c r="C5">
+        <v>20</v>
+      </c>
+      <c r="D5">
+        <v>15</v>
+      </c>
+      <c r="E5">
+        <v>10000</v>
+      </c>
+      <c r="F5">
+        <v>1000</v>
+      </c>
+      <c r="G5" t="str">
+        <v/>
+      </c>
+      <c r="H5" t="str">
+        <v>Precio y stock en gramos</v>
+      </c>
+      <c r="I5" t="str">
+        <v>si</v>
+      </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:H4"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:I5"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>